<commit_message>
Fixing bug - no impacts on published numbers.
</commit_message>
<xml_diff>
--- a/data/00_auxiliary/concordances/deflators_and_io.xlsx
+++ b/data/00_auxiliary/concordances/deflators_and_io.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kajwanr\Projects\cafean_python\data\auxiliary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kajwa\work\code\cafean\data\00_auxiliary\concordances\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27AC8E09-3A20-43D3-A4B5-F063EA8D3876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6118124B-3DC6-4091-95BD-ABA6960A6B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2010" windowWidth="25950" windowHeight="15300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7995" yWindow="3870" windowWidth="23085" windowHeight="13950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="domestic" sheetId="1" r:id="rId1"/>
@@ -1506,201 +1506,71 @@
   <autoFilter ref="A1:BN67" xr:uid="{845D890C-855F-4957-A489-5D3D5AE34AB9}"/>
   <tableColumns count="66">
     <tableColumn id="1" xr3:uid="{041D4FC4-EDE5-4874-9C02-DB0FB76C1FD5}" name="category" dataDxfId="203" totalsRowDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{0D70645A-F787-4E80-A755-AAD25D17AB01}" name="Products of agriculture, hunting and related services" totalsRowFunction="custom" dataDxfId="202" totalsRowDxfId="64">
-      <totalsRowFormula>SUM(Table1[Products of agriculture, hunting and related services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{2C6D528C-6C6F-44DE-A36F-8F9D829FD6D6}" name="Products of forestry, logging and related services" totalsRowFunction="custom" dataDxfId="201" totalsRowDxfId="63">
-      <totalsRowFormula>SUM(Table1[Products of forestry, logging and related services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="4" xr3:uid="{DA366293-0F21-4209-8C89-54345023ADD9}" name="Fish and other fishing products; aquaculture products; support services to fishing" totalsRowFunction="custom" dataDxfId="200" totalsRowDxfId="62">
-      <totalsRowFormula>SUM(Table1[Fish and other fishing products; aquaculture products; support services to fishing])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="5" xr3:uid="{513C757E-9854-4962-A860-84BA9F56011A}" name="Mining and quarrying" totalsRowFunction="custom" dataDxfId="199" totalsRowDxfId="61">
-      <totalsRowFormula>SUM(Table1[Mining and quarrying])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{215FBC7D-D908-4A65-AEE9-630D5E5BB135}" name="Food products, beverages and tobacco products" totalsRowFunction="custom" dataDxfId="198" totalsRowDxfId="60">
-      <totalsRowFormula>SUM(Table1[Food products, beverages and tobacco products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="7" xr3:uid="{98A487D2-8C26-44A7-BC74-C5C9C5D7A1E4}" name="Textiles, wearing apparel and leather products" totalsRowFunction="custom" dataDxfId="197" totalsRowDxfId="59">
-      <totalsRowFormula>SUM(Table1[Textiles, wearing apparel and leather products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="8" xr3:uid="{CB2D1204-3618-48FF-A212-CBAB845BEB77}" name="Wood and of products of wood and cork, except furniture; articles of straw and plaiting materials" totalsRowFunction="custom" dataDxfId="196" totalsRowDxfId="58">
-      <totalsRowFormula>SUM(Table1[Wood and of products of wood and cork, except furniture; articles of straw and plaiting materials])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="9" xr3:uid="{CA7301EA-5734-427C-96F0-26F03BDAA250}" name="Paper and paper products" totalsRowFunction="custom" dataDxfId="195" totalsRowDxfId="57">
-      <totalsRowFormula>SUM(Table1[Paper and paper products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="10" xr3:uid="{BFAB4CBE-CE7B-4683-8C5C-9162CD074C8F}" name="Printing and recording services" totalsRowFunction="custom" dataDxfId="194" totalsRowDxfId="56">
-      <totalsRowFormula>SUM(Table1[Printing and recording services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="11" xr3:uid="{87C59F62-D2FD-453F-A3EA-2F21A54A19A1}" name="Coke and refined petroleum products" totalsRowFunction="custom" dataDxfId="193" totalsRowDxfId="55">
-      <totalsRowFormula>SUM(Table1[Coke and refined petroleum products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="12" xr3:uid="{258B20E9-64AB-4F0D-A6FB-BB40C7A27CBE}" name="Chemicals and chemical products" totalsRowFunction="custom" dataDxfId="192" totalsRowDxfId="54">
-      <totalsRowFormula>SUM(Table1[Chemicals and chemical products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="13" xr3:uid="{1BAB6E11-6DF7-4F7E-9931-4F6CF2EC07DA}" name="Basic pharmaceutical products and pharmaceutical preparations" totalsRowFunction="custom" dataDxfId="191" totalsRowDxfId="53">
-      <totalsRowFormula>SUM(Table1[Basic pharmaceutical products and pharmaceutical preparations])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="14" xr3:uid="{F69AA913-7E91-4861-A78B-D564538676FA}" name="Rubber and plastics products" totalsRowFunction="custom" dataDxfId="190" totalsRowDxfId="52">
-      <totalsRowFormula>SUM(Table1[Rubber and plastics products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="15" xr3:uid="{445F0C2A-00C5-47B8-A9F6-13F417FC9AB2}" name="Other non-metallic mineral products" totalsRowFunction="custom" dataDxfId="189" totalsRowDxfId="51">
-      <totalsRowFormula>SUM(Table1[Other non-metallic mineral products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="16" xr3:uid="{91A85DA2-2C8F-4953-B3E6-6960504F9401}" name="Basic metals" totalsRowFunction="custom" dataDxfId="188" totalsRowDxfId="50">
-      <totalsRowFormula>SUM(Table1[Basic metals])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="17" xr3:uid="{49DBEF0F-5421-4029-BEA3-EA65A7D3EA42}" name="Fabricated metal products, except machinery and equipment" totalsRowFunction="custom" dataDxfId="187" totalsRowDxfId="49">
-      <totalsRowFormula>SUM(Table1[Fabricated metal products, except machinery and equipment])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="18" xr3:uid="{396369EF-3D2B-423F-AFF2-8C93644FF549}" name="Computer, electronic and optical products" totalsRowFunction="custom" dataDxfId="186" totalsRowDxfId="48">
-      <totalsRowFormula>SUM(Table1[Computer, electronic and optical products])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="19" xr3:uid="{74468C90-BADF-4311-A4B8-2A5008BC55F4}" name="Electrical equipment" totalsRowFunction="custom" dataDxfId="185" totalsRowDxfId="47">
-      <totalsRowFormula>SUM(Table1[Electrical equipment])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="20" xr3:uid="{23735639-5C02-4EE0-8977-CB0FA213AE3D}" name="Machinery and equipment n.e.c." totalsRowFunction="custom" dataDxfId="184" totalsRowDxfId="46">
-      <totalsRowFormula>SUM(Table1[Machinery and equipment n.e.c.])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="21" xr3:uid="{A8D89D91-46A8-4F2D-A45F-5D6158495116}" name="Motor vehicles, trailers and semi-trailers" totalsRowFunction="custom" dataDxfId="183" totalsRowDxfId="45">
-      <totalsRowFormula>SUM(Table1[Motor vehicles, trailers and semi-trailers])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="22" xr3:uid="{9654537C-CCD8-4B4F-85C5-41288E275699}" name="Other transport equipment" totalsRowFunction="custom" dataDxfId="182" totalsRowDxfId="44">
-      <totalsRowFormula>SUM(Table1[Other transport equipment])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="23" xr3:uid="{A7890C7F-6C72-4BC7-A9A2-18302AFF21AE}" name="Furniture; other manufactured goods" totalsRowFunction="custom" dataDxfId="181" totalsRowDxfId="43">
-      <totalsRowFormula>SUM(Table1[Furniture; other manufactured goods])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="24" xr3:uid="{A3CFBA80-D052-49CD-8FCB-7FF13C18387C}" name="Repair and installation services of machinery and equipment" totalsRowFunction="custom" dataDxfId="180" totalsRowDxfId="42">
-      <totalsRowFormula>SUM(Table1[Repair and installation services of machinery and equipment])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="25" xr3:uid="{363EBF14-B292-41E6-8D09-AB07532F81A6}" name="Electricity, gas, steam and air-conditioning" totalsRowFunction="custom" dataDxfId="179" totalsRowDxfId="41">
-      <totalsRowFormula>SUM(Table1[Electricity, gas, steam and air-conditioning])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="26" xr3:uid="{88454443-DB42-4594-B44B-CF0B702F072D}" name="Natural water; water treatment and supply services" totalsRowFunction="custom" dataDxfId="178" totalsRowDxfId="40">
-      <totalsRowFormula>SUM(Table1[Natural water; water treatment and supply services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="27" xr3:uid="{D2BCA1C4-F3BA-4A5C-A0C6-3D0665147D33}" name="Sewerage; waste collection, treatment and disposal activities; materials recovery; remediation activities and other waste management services" totalsRowFunction="custom" dataDxfId="177" totalsRowDxfId="39">
-      <totalsRowFormula>SUM(Table1[Sewerage; waste collection, treatment and disposal activities; materials recovery; remediation activities and other waste management services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="28" xr3:uid="{DA0E0183-8142-4094-A75D-78B44A20CFD9}" name="Constructions and construction works" totalsRowFunction="custom" dataDxfId="176" totalsRowDxfId="38">
-      <totalsRowFormula>SUM(Table1[Constructions and construction works])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="29" xr3:uid="{20EAFFDE-F70B-4A71-A4FC-24096435155D}" name="Wholesale and retail trade and repair services of motor vehicles and motorcycles" totalsRowFunction="custom" dataDxfId="175" totalsRowDxfId="37">
-      <totalsRowFormula>SUM(Table1[Wholesale and retail trade and repair services of motor vehicles and motorcycles])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="30" xr3:uid="{92975E3D-05B1-40A1-B290-D16339F9F9AE}" name="Wholesale trade services, except of motor vehicles and motorcycles" totalsRowFunction="custom" dataDxfId="174" totalsRowDxfId="36">
-      <totalsRowFormula>SUM(Table1[Wholesale trade services, except of motor vehicles and motorcycles])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="31" xr3:uid="{1C55A9CB-0BF6-4356-9086-F2C7CC9A8613}" name="Retail trade services, except of motor vehicles and motorcycles" totalsRowFunction="custom" dataDxfId="173" totalsRowDxfId="35">
-      <totalsRowFormula>SUM(Table1[Retail trade services, except of motor vehicles and motorcycles])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="32" xr3:uid="{EC43FDDE-EA76-495F-A949-6BFA5CF46840}" name="Land transport services and transport services via pipelines" totalsRowFunction="custom" dataDxfId="172" totalsRowDxfId="34">
-      <totalsRowFormula>SUM(Table1[Land transport services and transport services via pipelines])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="33" xr3:uid="{909DC159-8C24-4C10-9E9F-79B2125622F6}" name="Water transport services" totalsRowFunction="custom" dataDxfId="171" totalsRowDxfId="33">
-      <totalsRowFormula>SUM(Table1[Water transport services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="34" xr3:uid="{C3D3E0E8-4483-4A21-B124-FE531F9A30F3}" name="Air transport services" totalsRowFunction="custom" dataDxfId="170" totalsRowDxfId="32">
-      <totalsRowFormula>SUM(Table1[Air transport services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="35" xr3:uid="{25290538-8DB0-4A85-84F2-E282DE2DA17D}" name="Warehousing and support services for transportation" totalsRowFunction="custom" dataDxfId="169" totalsRowDxfId="31">
-      <totalsRowFormula>SUM(Table1[Warehousing and support services for transportation])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="36" xr3:uid="{3C35BA48-C73E-4A9B-A895-E000174861D5}" name="Postal and courier services" totalsRowFunction="custom" dataDxfId="168" totalsRowDxfId="30">
-      <totalsRowFormula>SUM(Table1[Postal and courier services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="37" xr3:uid="{9528762C-64CC-4B17-9689-E41F6AADE79E}" name="Accommodation and food services" totalsRowFunction="custom" dataDxfId="167" totalsRowDxfId="29">
-      <totalsRowFormula>SUM(Table1[Accommodation and food services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="38" xr3:uid="{56F56E0A-3601-477E-B9EC-9D10EC1F6605}" name="Publishing services" totalsRowFunction="custom" dataDxfId="166" totalsRowDxfId="28">
-      <totalsRowFormula>SUM(Table1[Publishing services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="39" xr3:uid="{85F07DE9-B42E-49EA-A28A-31ED037F8FC2}" name="Motion picture, video and television programme production services, sound recording and music publishing; programming and broadcasting services" totalsRowFunction="custom" dataDxfId="165" totalsRowDxfId="27">
-      <totalsRowFormula>SUM(Table1[Motion picture, video and television programme production services, sound recording and music publishing; programming and broadcasting services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="40" xr3:uid="{9FAE8999-3ADA-4B47-9636-BA39CF2A0F69}" name="Telecommunications services" totalsRowFunction="custom" dataDxfId="164" totalsRowDxfId="26">
-      <totalsRowFormula>SUM(Table1[Telecommunications services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="41" xr3:uid="{C3817EA6-1F76-471A-84D8-D31AF2C78177}" name="Computer programming, consultancy and related services; information services" totalsRowFunction="custom" dataDxfId="163" totalsRowDxfId="25">
-      <totalsRowFormula>SUM(Table1[Computer programming, consultancy and related services; information services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="42" xr3:uid="{EA5B36F0-2E0D-4AA1-884E-8F495E9ADD49}" name="Financial services, except insurance and pension funding" totalsRowFunction="custom" dataDxfId="162" totalsRowDxfId="24">
-      <totalsRowFormula>SUM(Table1[Financial services, except insurance and pension funding])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="43" xr3:uid="{3AB6BE01-0D26-49CB-9199-9D3C65E01601}" name="Insurance, reinsurance and pension funding services, except compulsory social security" totalsRowFunction="custom" dataDxfId="161" totalsRowDxfId="23">
-      <totalsRowFormula>SUM(Table1[Insurance, reinsurance and pension funding services, except compulsory social security])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="44" xr3:uid="{2FC6F85B-4D70-434C-AECA-23A0A85BE9FA}" name="Services auxiliary to financial services and insurance services" totalsRowFunction="custom" dataDxfId="160" totalsRowDxfId="22">
-      <totalsRowFormula>SUM(Table1[Services auxiliary to financial services and insurance services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="45" xr3:uid="{A5E41895-416B-4193-9E85-54E1AF3790B8}" name="Real estate services (excluding imputed rents)" totalsRowFunction="custom" dataDxfId="159" totalsRowDxfId="21">
-      <totalsRowFormula>SUM(Table1[Real estate services (excluding imputed rents)])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="46" xr3:uid="{4EF8E6D3-9BD8-4AE6-AB8E-17AD133B5770}" name="Imputed rents of owner-occupied dwellings" totalsRowFunction="custom" dataDxfId="158" totalsRowDxfId="20">
-      <totalsRowFormula>SUM(Table1[Imputed rents of owner-occupied dwellings])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="47" xr3:uid="{8374C4F9-BBF7-4765-8FED-08C6DD6E603C}" name="Legal and accounting services; services of head offices; management consulting services" totalsRowFunction="custom" dataDxfId="157" totalsRowDxfId="19">
-      <totalsRowFormula>SUM(Table1[Legal and accounting services; services of head offices; management consulting services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="48" xr3:uid="{A17E457A-9B08-4B43-9573-CD82B7EF18DC}" name="Architectural and engineering services; technical testing and analysis services" totalsRowFunction="custom" dataDxfId="156" totalsRowDxfId="18">
-      <totalsRowFormula>SUM(Table1[Architectural and engineering services; technical testing and analysis services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="49" xr3:uid="{8382A72D-F4DB-44CF-82C4-5BBA272B7938}" name="Scientific research and development services" totalsRowFunction="custom" dataDxfId="155" totalsRowDxfId="17">
-      <totalsRowFormula>SUM(Table1[Scientific research and development services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="50" xr3:uid="{0C56D9F2-EF9E-47B1-AD71-75EAB6ED7F2E}" name="Advertising and market research services" totalsRowFunction="custom" dataDxfId="154" totalsRowDxfId="16">
-      <totalsRowFormula>SUM(Table1[Advertising and market research services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="51" xr3:uid="{CF6D1A86-3EA9-437A-86A4-886A5E8EFD92}" name="Other professional, scientific and technical services; veterinary services" totalsRowFunction="custom" dataDxfId="153" totalsRowDxfId="15">
-      <totalsRowFormula>SUM(Table1[Other professional, scientific and technical services; veterinary services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="52" xr3:uid="{638BC058-0A84-45A4-B668-5E08C8F9CA5B}" name="Rental and leasing services" totalsRowFunction="custom" dataDxfId="152" totalsRowDxfId="14">
-      <totalsRowFormula>SUM(Table1[Rental and leasing services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="53" xr3:uid="{B884F516-2EDA-407B-B88A-EE11D422E465}" name="Employment services" totalsRowFunction="custom" dataDxfId="151" totalsRowDxfId="13">
-      <totalsRowFormula>SUM(Table1[Employment services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="54" xr3:uid="{8832C7A0-C816-4BD1-BC12-B2C910BA984D}" name="Travel agency, tour operator and other reservation services and related services" totalsRowFunction="custom" dataDxfId="150" totalsRowDxfId="12">
-      <totalsRowFormula>SUM(Table1[Travel agency, tour operator and other reservation services and related services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="55" xr3:uid="{09F9C5CF-0A57-40AF-89EC-8ACC0CAA59F9}" name="Security and investigation services; services to buildings and landscape; office administrative, office support and other business support services" totalsRowFunction="custom" dataDxfId="149" totalsRowDxfId="11">
-      <totalsRowFormula>SUM(Table1[Security and investigation services; services to buildings and landscape; office administrative, office support and other business support services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="56" xr3:uid="{C0BF15BB-A475-4D3E-8203-E41873DA8403}" name="Public administration and defence services; compulsory social security services" totalsRowFunction="custom" dataDxfId="148" totalsRowDxfId="10">
-      <totalsRowFormula>SUM(Table1[Public administration and defence services; compulsory social security services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="57" xr3:uid="{52FA0BDF-714F-47C2-A8B5-EC07057CBF83}" name="Education services" totalsRowFunction="custom" dataDxfId="147" totalsRowDxfId="9">
-      <totalsRowFormula>SUM(Table1[Education services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="58" xr3:uid="{DD084E21-D158-4770-9A9C-C86F9AB6A72D}" name="Human health services" totalsRowFunction="custom" dataDxfId="146" totalsRowDxfId="8">
-      <totalsRowFormula>SUM(Table1[Human health services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="59" xr3:uid="{6AEF7772-1A7E-4C35-9FF8-9926E0F1BF96}" name="Social work services" totalsRowFunction="custom" dataDxfId="145" totalsRowDxfId="7">
-      <totalsRowFormula>SUM(Table1[Social work services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="60" xr3:uid="{A71F8B02-F899-459C-BF78-529E37E46FEC}" name="Creative, arts and entertainment services; library, archive, museum and other cultural services; gambling and betting services" totalsRowFunction="custom" dataDxfId="144" totalsRowDxfId="6">
-      <totalsRowFormula>SUM(Table1[Creative, arts and entertainment services; library, archive, museum and other cultural services; gambling and betting services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="61" xr3:uid="{8797E9B4-E06E-4015-ADD7-AA5911289AB9}" name="Sporting services and amusement and recreation services" totalsRowFunction="custom" dataDxfId="143" totalsRowDxfId="5">
-      <totalsRowFormula>SUM(Table1[Sporting services and amusement and recreation services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="62" xr3:uid="{FA078E95-1EC9-469A-9343-63723F6D25E3}" name="Services furnished by membership organisations" totalsRowFunction="custom" dataDxfId="142" totalsRowDxfId="4">
-      <totalsRowFormula>SUM(Table1[Services furnished by membership organisations])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="63" xr3:uid="{1C6C1515-7BD3-4E32-8C4C-605437FB428C}" name="Repair services of computers and personal and household goods" totalsRowFunction="custom" dataDxfId="141" totalsRowDxfId="3">
-      <totalsRowFormula>SUM(Table1[Repair services of computers and personal and household goods])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="64" xr3:uid="{47748F96-37A8-4A6C-8AA3-A17FB171CFB6}" name="Other personal services" totalsRowFunction="custom" dataDxfId="140" totalsRowDxfId="2">
-      <totalsRowFormula>SUM(Table1[Other personal services])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="65" xr3:uid="{86F260B3-068A-4B81-807A-C55DEB1055B5}" name="Services of households as employers; undifferentiated goods and services produced by households for own use" totalsRowFunction="custom" dataDxfId="139" totalsRowDxfId="1">
-      <totalsRowFormula>SUM(Table1[Services of households as employers; undifferentiated goods and services produced by households for own use])</totalsRowFormula>
-    </tableColumn>
-    <tableColumn id="66" xr3:uid="{5432E62E-0159-4FDB-A462-F51555DB9C07}" name="Services provided by extraterritorial organisations and bodies" totalsRowFunction="custom" dataDxfId="138" totalsRowDxfId="0">
-      <totalsRowFormula>SUM(Table1[Services provided by extraterritorial organisations and bodies])</totalsRowFormula>
-    </tableColumn>
+    <tableColumn id="2" xr3:uid="{0D70645A-F787-4E80-A755-AAD25D17AB01}" name="Products of agriculture, hunting and related services" dataDxfId="202" totalsRowDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{2C6D528C-6C6F-44DE-A36F-8F9D829FD6D6}" name="Products of forestry, logging and related services" dataDxfId="201" totalsRowDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{DA366293-0F21-4209-8C89-54345023ADD9}" name="Fish and other fishing products; aquaculture products; support services to fishing" dataDxfId="200" totalsRowDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{513C757E-9854-4962-A860-84BA9F56011A}" name="Mining and quarrying" dataDxfId="199" totalsRowDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{215FBC7D-D908-4A65-AEE9-630D5E5BB135}" name="Food products, beverages and tobacco products" dataDxfId="198" totalsRowDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{98A487D2-8C26-44A7-BC74-C5C9C5D7A1E4}" name="Textiles, wearing apparel and leather products" dataDxfId="197" totalsRowDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{CB2D1204-3618-48FF-A212-CBAB845BEB77}" name="Wood and of products of wood and cork, except furniture; articles of straw and plaiting materials" dataDxfId="196" totalsRowDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{CA7301EA-5734-427C-96F0-26F03BDAA250}" name="Paper and paper products" dataDxfId="195" totalsRowDxfId="57"/>
+    <tableColumn id="10" xr3:uid="{BFAB4CBE-CE7B-4683-8C5C-9162CD074C8F}" name="Printing and recording services" dataDxfId="194" totalsRowDxfId="56"/>
+    <tableColumn id="11" xr3:uid="{87C59F62-D2FD-453F-A3EA-2F21A54A19A1}" name="Coke and refined petroleum products" dataDxfId="193" totalsRowDxfId="55"/>
+    <tableColumn id="12" xr3:uid="{258B20E9-64AB-4F0D-A6FB-BB40C7A27CBE}" name="Chemicals and chemical products" dataDxfId="192" totalsRowDxfId="54"/>
+    <tableColumn id="13" xr3:uid="{1BAB6E11-6DF7-4F7E-9931-4F6CF2EC07DA}" name="Basic pharmaceutical products and pharmaceutical preparations" dataDxfId="191" totalsRowDxfId="53"/>
+    <tableColumn id="14" xr3:uid="{F69AA913-7E91-4861-A78B-D564538676FA}" name="Rubber and plastics products" dataDxfId="190" totalsRowDxfId="52"/>
+    <tableColumn id="15" xr3:uid="{445F0C2A-00C5-47B8-A9F6-13F417FC9AB2}" name="Other non-metallic mineral products" dataDxfId="189" totalsRowDxfId="51"/>
+    <tableColumn id="16" xr3:uid="{91A85DA2-2C8F-4953-B3E6-6960504F9401}" name="Basic metals" dataDxfId="188" totalsRowDxfId="50"/>
+    <tableColumn id="17" xr3:uid="{49DBEF0F-5421-4029-BEA3-EA65A7D3EA42}" name="Fabricated metal products, except machinery and equipment" dataDxfId="187" totalsRowDxfId="49"/>
+    <tableColumn id="18" xr3:uid="{396369EF-3D2B-423F-AFF2-8C93644FF549}" name="Computer, electronic and optical products" dataDxfId="186" totalsRowDxfId="48"/>
+    <tableColumn id="19" xr3:uid="{74468C90-BADF-4311-A4B8-2A5008BC55F4}" name="Electrical equipment" dataDxfId="185" totalsRowDxfId="47"/>
+    <tableColumn id="20" xr3:uid="{23735639-5C02-4EE0-8977-CB0FA213AE3D}" name="Machinery and equipment n.e.c." dataDxfId="184" totalsRowDxfId="46"/>
+    <tableColumn id="21" xr3:uid="{A8D89D91-46A8-4F2D-A45F-5D6158495116}" name="Motor vehicles, trailers and semi-trailers" dataDxfId="183" totalsRowDxfId="45"/>
+    <tableColumn id="22" xr3:uid="{9654537C-CCD8-4B4F-85C5-41288E275699}" name="Other transport equipment" dataDxfId="182" totalsRowDxfId="44"/>
+    <tableColumn id="23" xr3:uid="{A7890C7F-6C72-4BC7-A9A2-18302AFF21AE}" name="Furniture; other manufactured goods" dataDxfId="181" totalsRowDxfId="43"/>
+    <tableColumn id="24" xr3:uid="{A3CFBA80-D052-49CD-8FCB-7FF13C18387C}" name="Repair and installation services of machinery and equipment" dataDxfId="180" totalsRowDxfId="42"/>
+    <tableColumn id="25" xr3:uid="{363EBF14-B292-41E6-8D09-AB07532F81A6}" name="Electricity, gas, steam and air-conditioning" dataDxfId="179" totalsRowDxfId="41"/>
+    <tableColumn id="26" xr3:uid="{88454443-DB42-4594-B44B-CF0B702F072D}" name="Natural water; water treatment and supply services" dataDxfId="178" totalsRowDxfId="40"/>
+    <tableColumn id="27" xr3:uid="{D2BCA1C4-F3BA-4A5C-A0C6-3D0665147D33}" name="Sewerage; waste collection, treatment and disposal activities; materials recovery; remediation activities and other waste management services" dataDxfId="177" totalsRowDxfId="39"/>
+    <tableColumn id="28" xr3:uid="{DA0E0183-8142-4094-A75D-78B44A20CFD9}" name="Constructions and construction works" dataDxfId="176" totalsRowDxfId="38"/>
+    <tableColumn id="29" xr3:uid="{20EAFFDE-F70B-4A71-A4FC-24096435155D}" name="Wholesale and retail trade and repair services of motor vehicles and motorcycles" dataDxfId="175" totalsRowDxfId="37"/>
+    <tableColumn id="30" xr3:uid="{92975E3D-05B1-40A1-B290-D16339F9F9AE}" name="Wholesale trade services, except of motor vehicles and motorcycles" dataDxfId="174" totalsRowDxfId="36"/>
+    <tableColumn id="31" xr3:uid="{1C55A9CB-0BF6-4356-9086-F2C7CC9A8613}" name="Retail trade services, except of motor vehicles and motorcycles" dataDxfId="173" totalsRowDxfId="35"/>
+    <tableColumn id="32" xr3:uid="{EC43FDDE-EA76-495F-A949-6BFA5CF46840}" name="Land transport services and transport services via pipelines" dataDxfId="172" totalsRowDxfId="34"/>
+    <tableColumn id="33" xr3:uid="{909DC159-8C24-4C10-9E9F-79B2125622F6}" name="Water transport services" dataDxfId="171" totalsRowDxfId="33"/>
+    <tableColumn id="34" xr3:uid="{C3D3E0E8-4483-4A21-B124-FE531F9A30F3}" name="Air transport services" dataDxfId="170" totalsRowDxfId="32"/>
+    <tableColumn id="35" xr3:uid="{25290538-8DB0-4A85-84F2-E282DE2DA17D}" name="Warehousing and support services for transportation" dataDxfId="169" totalsRowDxfId="31"/>
+    <tableColumn id="36" xr3:uid="{3C35BA48-C73E-4A9B-A895-E000174861D5}" name="Postal and courier services" dataDxfId="168" totalsRowDxfId="30"/>
+    <tableColumn id="37" xr3:uid="{9528762C-64CC-4B17-9689-E41F6AADE79E}" name="Accommodation and food services" dataDxfId="167" totalsRowDxfId="29"/>
+    <tableColumn id="38" xr3:uid="{56F56E0A-3601-477E-B9EC-9D10EC1F6605}" name="Publishing services" dataDxfId="166" totalsRowDxfId="28"/>
+    <tableColumn id="39" xr3:uid="{85F07DE9-B42E-49EA-A28A-31ED037F8FC2}" name="Motion picture, video and television programme production services, sound recording and music publishing; programming and broadcasting services" dataDxfId="165" totalsRowDxfId="27"/>
+    <tableColumn id="40" xr3:uid="{9FAE8999-3ADA-4B47-9636-BA39CF2A0F69}" name="Telecommunications services" dataDxfId="164" totalsRowDxfId="26"/>
+    <tableColumn id="41" xr3:uid="{C3817EA6-1F76-471A-84D8-D31AF2C78177}" name="Computer programming, consultancy and related services; information services" dataDxfId="163" totalsRowDxfId="25"/>
+    <tableColumn id="42" xr3:uid="{EA5B36F0-2E0D-4AA1-884E-8F495E9ADD49}" name="Financial services, except insurance and pension funding" dataDxfId="162" totalsRowDxfId="24"/>
+    <tableColumn id="43" xr3:uid="{3AB6BE01-0D26-49CB-9199-9D3C65E01601}" name="Insurance, reinsurance and pension funding services, except compulsory social security" dataDxfId="161" totalsRowDxfId="23"/>
+    <tableColumn id="44" xr3:uid="{2FC6F85B-4D70-434C-AECA-23A0A85BE9FA}" name="Services auxiliary to financial services and insurance services" dataDxfId="160" totalsRowDxfId="22"/>
+    <tableColumn id="45" xr3:uid="{A5E41895-416B-4193-9E85-54E1AF3790B8}" name="Real estate services (excluding imputed rents)" dataDxfId="159" totalsRowDxfId="21"/>
+    <tableColumn id="46" xr3:uid="{4EF8E6D3-9BD8-4AE6-AB8E-17AD133B5770}" name="Imputed rents of owner-occupied dwellings" dataDxfId="158" totalsRowDxfId="20"/>
+    <tableColumn id="47" xr3:uid="{8374C4F9-BBF7-4765-8FED-08C6DD6E603C}" name="Legal and accounting services; services of head offices; management consulting services" dataDxfId="157" totalsRowDxfId="19"/>
+    <tableColumn id="48" xr3:uid="{A17E457A-9B08-4B43-9573-CD82B7EF18DC}" name="Architectural and engineering services; technical testing and analysis services" dataDxfId="156" totalsRowDxfId="18"/>
+    <tableColumn id="49" xr3:uid="{8382A72D-F4DB-44CF-82C4-5BBA272B7938}" name="Scientific research and development services" dataDxfId="155" totalsRowDxfId="17"/>
+    <tableColumn id="50" xr3:uid="{0C56D9F2-EF9E-47B1-AD71-75EAB6ED7F2E}" name="Advertising and market research services" dataDxfId="154" totalsRowDxfId="16"/>
+    <tableColumn id="51" xr3:uid="{CF6D1A86-3EA9-437A-86A4-886A5E8EFD92}" name="Other professional, scientific and technical services; veterinary services" dataDxfId="153" totalsRowDxfId="15"/>
+    <tableColumn id="52" xr3:uid="{638BC058-0A84-45A4-B668-5E08C8F9CA5B}" name="Rental and leasing services" dataDxfId="152" totalsRowDxfId="14"/>
+    <tableColumn id="53" xr3:uid="{B884F516-2EDA-407B-B88A-EE11D422E465}" name="Employment services" dataDxfId="151" totalsRowDxfId="13"/>
+    <tableColumn id="54" xr3:uid="{8832C7A0-C816-4BD1-BC12-B2C910BA984D}" name="Travel agency, tour operator and other reservation services and related services" dataDxfId="150" totalsRowDxfId="12"/>
+    <tableColumn id="55" xr3:uid="{09F9C5CF-0A57-40AF-89EC-8ACC0CAA59F9}" name="Security and investigation services; services to buildings and landscape; office administrative, office support and other business support services" dataDxfId="149" totalsRowDxfId="11"/>
+    <tableColumn id="56" xr3:uid="{C0BF15BB-A475-4D3E-8203-E41873DA8403}" name="Public administration and defence services; compulsory social security services" dataDxfId="148" totalsRowDxfId="10"/>
+    <tableColumn id="57" xr3:uid="{52FA0BDF-714F-47C2-A8B5-EC07057CBF83}" name="Education services" dataDxfId="147" totalsRowDxfId="9"/>
+    <tableColumn id="58" xr3:uid="{DD084E21-D158-4770-9A9C-C86F9AB6A72D}" name="Human health services" dataDxfId="146" totalsRowDxfId="8"/>
+    <tableColumn id="59" xr3:uid="{6AEF7772-1A7E-4C35-9FF8-9926E0F1BF96}" name="Social work services" dataDxfId="145" totalsRowDxfId="7"/>
+    <tableColumn id="60" xr3:uid="{A71F8B02-F899-459C-BF78-529E37E46FEC}" name="Creative, arts and entertainment services; library, archive, museum and other cultural services; gambling and betting services" dataDxfId="144" totalsRowDxfId="6"/>
+    <tableColumn id="61" xr3:uid="{8797E9B4-E06E-4015-ADD7-AA5911289AB9}" name="Sporting services and amusement and recreation services" dataDxfId="143" totalsRowDxfId="5"/>
+    <tableColumn id="62" xr3:uid="{FA078E95-1EC9-469A-9343-63723F6D25E3}" name="Services furnished by membership organisations" dataDxfId="142" totalsRowDxfId="4"/>
+    <tableColumn id="63" xr3:uid="{1C6C1515-7BD3-4E32-8C4C-605437FB428C}" name="Repair services of computers and personal and household goods" dataDxfId="141" totalsRowDxfId="3"/>
+    <tableColumn id="64" xr3:uid="{47748F96-37A8-4A6C-8AA3-A17FB171CFB6}" name="Other personal services" dataDxfId="140" totalsRowDxfId="2"/>
+    <tableColumn id="65" xr3:uid="{86F260B3-068A-4B81-807A-C55DEB1055B5}" name="Services of households as employers; undifferentiated goods and services produced by households for own use" dataDxfId="139" totalsRowDxfId="1"/>
+    <tableColumn id="66" xr3:uid="{5432E62E-0159-4FDB-A462-F51555DB9C07}" name="Services provided by extraterritorial organisations and bodies" dataDxfId="138" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15475,266 +15345,71 @@
     </row>
     <row r="68" spans="1:66" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="1">
-        <f>SUM(Table1[Products of agriculture, hunting and related services])</f>
-        <v>1</v>
-      </c>
-      <c r="C68" s="1">
-        <f>SUM(Table1[Products of forestry, logging and related services])</f>
-        <v>1</v>
-      </c>
-      <c r="D68" s="1">
-        <f>SUM(Table1[Fish and other fishing products; aquaculture products; support services to fishing])</f>
-        <v>2</v>
-      </c>
-      <c r="E68" s="1">
-        <f>SUM(Table1[Mining and quarrying])</f>
-        <v>3</v>
-      </c>
-      <c r="F68" s="1">
-        <f>SUM(Table1[Food products, beverages and tobacco products])</f>
-        <v>1</v>
-      </c>
-      <c r="G68" s="1">
-        <f>SUM(Table1[Textiles, wearing apparel and leather products])</f>
-        <v>1</v>
-      </c>
-      <c r="H68" s="1">
-        <f>SUM(Table1[Wood and of products of wood and cork, except furniture; articles of straw and plaiting materials])</f>
-        <v>1</v>
-      </c>
-      <c r="I68" s="1">
-        <f>SUM(Table1[Paper and paper products])</f>
-        <v>1</v>
-      </c>
-      <c r="J68" s="1">
-        <f>SUM(Table1[Printing and recording services])</f>
-        <v>1</v>
-      </c>
-      <c r="K68" s="1">
-        <f>SUM(Table1[Coke and refined petroleum products])</f>
-        <v>1</v>
-      </c>
-      <c r="L68" s="1">
-        <f>SUM(Table1[Chemicals and chemical products])</f>
-        <v>1</v>
-      </c>
-      <c r="M68" s="1">
-        <f>SUM(Table1[Basic pharmaceutical products and pharmaceutical preparations])</f>
-        <v>1</v>
-      </c>
-      <c r="N68" s="1">
-        <f>SUM(Table1[Rubber and plastics products])</f>
-        <v>1</v>
-      </c>
-      <c r="O68" s="1">
-        <f>SUM(Table1[Other non-metallic mineral products])</f>
-        <v>1</v>
-      </c>
-      <c r="P68" s="1">
-        <f>SUM(Table1[Basic metals])</f>
-        <v>1</v>
-      </c>
-      <c r="Q68" s="1">
-        <f>SUM(Table1[Fabricated metal products, except machinery and equipment])</f>
-        <v>1</v>
-      </c>
-      <c r="R68" s="1">
-        <f>SUM(Table1[Computer, electronic and optical products])</f>
-        <v>1</v>
-      </c>
-      <c r="S68" s="1">
-        <f>SUM(Table1[Electrical equipment])</f>
-        <v>1</v>
-      </c>
-      <c r="T68" s="1">
-        <f>SUM(Table1[Machinery and equipment n.e.c.])</f>
-        <v>1</v>
-      </c>
-      <c r="U68" s="1">
-        <f>SUM(Table1[Motor vehicles, trailers and semi-trailers])</f>
-        <v>1</v>
-      </c>
-      <c r="V68" s="1">
-        <f>SUM(Table1[Other transport equipment])</f>
-        <v>1</v>
-      </c>
-      <c r="W68" s="1">
-        <f>SUM(Table1[Furniture; other manufactured goods])</f>
-        <v>1</v>
-      </c>
-      <c r="X68" s="1">
-        <f>SUM(Table1[Repair and installation services of machinery and equipment])</f>
-        <v>1</v>
-      </c>
-      <c r="Y68" s="1">
-        <f>SUM(Table1[Electricity, gas, steam and air-conditioning])</f>
-        <v>1</v>
-      </c>
-      <c r="Z68" s="1">
-        <f>SUM(Table1[Natural water; water treatment and supply services])</f>
-        <v>1</v>
-      </c>
-      <c r="AA68" s="1">
-        <f>SUM(Table1[Sewerage; waste collection, treatment and disposal activities; materials recovery; remediation activities and other waste management services])</f>
-        <v>1</v>
-      </c>
-      <c r="AB68" s="1">
-        <f>SUM(Table1[Constructions and construction works])</f>
-        <v>1</v>
-      </c>
-      <c r="AC68" s="1">
-        <f>SUM(Table1[Wholesale and retail trade and repair services of motor vehicles and motorcycles])</f>
-        <v>1</v>
-      </c>
-      <c r="AD68" s="1">
-        <f>SUM(Table1[Wholesale trade services, except of motor vehicles and motorcycles])</f>
-        <v>1</v>
-      </c>
-      <c r="AE68" s="1">
-        <f>SUM(Table1[Retail trade services, except of motor vehicles and motorcycles])</f>
-        <v>1</v>
-      </c>
-      <c r="AF68" s="1">
-        <f>SUM(Table1[Land transport services and transport services via pipelines])</f>
-        <v>2</v>
-      </c>
-      <c r="AG68" s="1">
-        <f>SUM(Table1[Water transport services])</f>
-        <v>2</v>
-      </c>
-      <c r="AH68" s="1">
-        <f>SUM(Table1[Air transport services])</f>
-        <v>1</v>
-      </c>
-      <c r="AI68" s="1">
-        <f>SUM(Table1[Warehousing and support services for transportation])</f>
-        <v>1</v>
-      </c>
-      <c r="AJ68" s="1">
-        <f>SUM(Table1[Postal and courier services])</f>
-        <v>1</v>
-      </c>
-      <c r="AK68" s="1">
-        <f>SUM(Table1[Accommodation and food services])</f>
-        <v>1</v>
-      </c>
-      <c r="AL68" s="1">
-        <f>SUM(Table1[Publishing services])</f>
-        <v>1</v>
-      </c>
-      <c r="AM68" s="1">
-        <f>SUM(Table1[Motion picture, video and television programme production services, sound recording and music publishing; programming and broadcasting services])</f>
-        <v>1</v>
-      </c>
-      <c r="AN68" s="1">
-        <f>SUM(Table1[Telecommunications services])</f>
-        <v>1</v>
-      </c>
-      <c r="AO68" s="1">
-        <f>SUM(Table1[Computer programming, consultancy and related services; information services])</f>
-        <v>1</v>
-      </c>
-      <c r="AP68" s="1">
-        <f>SUM(Table1[Financial services, except insurance and pension funding])</f>
-        <v>1</v>
-      </c>
-      <c r="AQ68" s="1">
-        <f>SUM(Table1[Insurance, reinsurance and pension funding services, except compulsory social security])</f>
-        <v>1</v>
-      </c>
-      <c r="AR68" s="1">
-        <f>SUM(Table1[Services auxiliary to financial services and insurance services])</f>
-        <v>1</v>
-      </c>
-      <c r="AS68" s="1">
-        <f>SUM(Table1[Real estate services (excluding imputed rents)])</f>
-        <v>1</v>
-      </c>
-      <c r="AT68" s="1">
-        <f>SUM(Table1[Imputed rents of owner-occupied dwellings])</f>
-        <v>1</v>
-      </c>
-      <c r="AU68" s="1">
-        <f>SUM(Table1[Legal and accounting services; services of head offices; management consulting services])</f>
-        <v>1</v>
-      </c>
-      <c r="AV68" s="1">
-        <f>SUM(Table1[Architectural and engineering services; technical testing and analysis services])</f>
-        <v>1</v>
-      </c>
-      <c r="AW68" s="1">
-        <f>SUM(Table1[Scientific research and development services])</f>
-        <v>1</v>
-      </c>
-      <c r="AX68" s="1">
-        <f>SUM(Table1[Advertising and market research services])</f>
-        <v>1</v>
-      </c>
-      <c r="AY68" s="1">
-        <f>SUM(Table1[Other professional, scientific and technical services; veterinary services])</f>
-        <v>1</v>
-      </c>
-      <c r="AZ68" s="1">
-        <f>SUM(Table1[Rental and leasing services])</f>
-        <v>1</v>
-      </c>
-      <c r="BA68" s="1">
-        <f>SUM(Table1[Employment services])</f>
-        <v>1</v>
-      </c>
-      <c r="BB68" s="1">
-        <f>SUM(Table1[Travel agency, tour operator and other reservation services and related services])</f>
-        <v>1</v>
-      </c>
-      <c r="BC68" s="1">
-        <f>SUM(Table1[Security and investigation services; services to buildings and landscape; office administrative, office support and other business support services])</f>
-        <v>1</v>
-      </c>
-      <c r="BD68" s="1">
-        <f>SUM(Table1[Public administration and defence services; compulsory social security services])</f>
-        <v>1</v>
-      </c>
-      <c r="BE68" s="1">
-        <f>SUM(Table1[Education services])</f>
-        <v>1</v>
-      </c>
-      <c r="BF68" s="1">
-        <f>SUM(Table1[Human health services])</f>
-        <v>1</v>
-      </c>
-      <c r="BG68" s="1">
-        <f>SUM(Table1[Social work services])</f>
-        <v>1</v>
-      </c>
-      <c r="BH68" s="1">
-        <f>SUM(Table1[Creative, arts and entertainment services; library, archive, museum and other cultural services; gambling and betting services])</f>
-        <v>1</v>
-      </c>
-      <c r="BI68" s="1">
-        <f>SUM(Table1[Sporting services and amusement and recreation services])</f>
-        <v>1</v>
-      </c>
-      <c r="BJ68" s="1">
-        <f>SUM(Table1[Services furnished by membership organisations])</f>
-        <v>1</v>
-      </c>
-      <c r="BK68" s="1">
-        <f>SUM(Table1[Repair services of computers and personal and household goods])</f>
-        <v>1</v>
-      </c>
-      <c r="BL68" s="1">
-        <f>SUM(Table1[Other personal services])</f>
-        <v>1</v>
-      </c>
-      <c r="BM68" s="1">
-        <f>SUM(Table1[Services of households as employers; undifferentiated goods and services produced by households for own use])</f>
-        <v>1</v>
-      </c>
-      <c r="BN68" s="1">
-        <f>SUM(Table1[Services provided by extraterritorial organisations and bodies])</f>
-        <v>1</v>
-      </c>
+      <c r="B68" s="1"/>
+      <c r="C68" s="1"/>
+      <c r="D68" s="1"/>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1"/>
+      <c r="G68" s="1"/>
+      <c r="H68" s="1"/>
+      <c r="I68" s="1"/>
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+      <c r="L68" s="1"/>
+      <c r="M68" s="1"/>
+      <c r="N68" s="1"/>
+      <c r="O68" s="1"/>
+      <c r="P68" s="1"/>
+      <c r="Q68" s="1"/>
+      <c r="R68" s="1"/>
+      <c r="S68" s="1"/>
+      <c r="T68" s="1"/>
+      <c r="U68" s="1"/>
+      <c r="V68" s="1"/>
+      <c r="W68" s="1"/>
+      <c r="X68" s="1"/>
+      <c r="Y68" s="1"/>
+      <c r="Z68" s="1"/>
+      <c r="AA68" s="1"/>
+      <c r="AB68" s="1"/>
+      <c r="AC68" s="1"/>
+      <c r="AD68" s="1"/>
+      <c r="AE68" s="1"/>
+      <c r="AF68" s="1"/>
+      <c r="AG68" s="1"/>
+      <c r="AH68" s="1"/>
+      <c r="AI68" s="1"/>
+      <c r="AJ68" s="1"/>
+      <c r="AK68" s="1"/>
+      <c r="AL68" s="1"/>
+      <c r="AM68" s="1"/>
+      <c r="AN68" s="1"/>
+      <c r="AO68" s="1"/>
+      <c r="AP68" s="1"/>
+      <c r="AQ68" s="1"/>
+      <c r="AR68" s="1"/>
+      <c r="AS68" s="1"/>
+      <c r="AT68" s="1"/>
+      <c r="AU68" s="1"/>
+      <c r="AV68" s="1"/>
+      <c r="AW68" s="1"/>
+      <c r="AX68" s="1"/>
+      <c r="AY68" s="1"/>
+      <c r="AZ68" s="1"/>
+      <c r="BA68" s="1"/>
+      <c r="BB68" s="1"/>
+      <c r="BC68" s="1"/>
+      <c r="BD68" s="1"/>
+      <c r="BE68" s="1"/>
+      <c r="BF68" s="1"/>
+      <c r="BG68" s="1"/>
+      <c r="BH68" s="1"/>
+      <c r="BI68" s="1"/>
+      <c r="BJ68" s="1"/>
+      <c r="BK68" s="1"/>
+      <c r="BL68" s="1"/>
+      <c r="BM68" s="1"/>
+      <c r="BN68" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:BN67">

</xml_diff>